<commit_message>
feat: add academic fields to members and update related queries
- Updated CSV template for importing members to include faculty, study program, and cohort year.
- Modified SQL queries and Go structs to accommodate new member fields (faculty, study program, cohort year).
- Enhanced member import functionality to handle new fields.
- Updated organization tree and member division queries to include academic information.
- Added tests to ensure JSON serialization of raw JSONB fields.
</commit_message>
<xml_diff>
--- a/docs/templates/template_import_members.xlsx
+++ b/docs/templates/template_import_members.xlsx
@@ -160,7 +160,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">period_start
+          <t xml:space="preserve">faculty
 </t>
         </r>
         <r>
@@ -170,7 +170,7 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">WAJIB DIISI. Tahun mulai kepengurusan, empat digit.</t>
+          <t xml:space="preserve">Fakultas anggota.</t>
         </r>
       </text>
     </comment>
@@ -182,7 +182,7 @@
             <b val="1"/>
             <color/>
           </rPr>
-          <t xml:space="preserve">period_end
+          <t xml:space="preserve">study_program
 </t>
         </r>
         <r>
@@ -192,11 +192,77 @@
             <color indexed="81"/>
             <sz val="9"/>
           </rPr>
-          <t xml:space="preserve">WAJIB DIISI. Tahun akhir kepengurusan, empat digit.</t>
+          <t xml:space="preserve">Program studi anggota.</t>
         </r>
       </text>
     </comment>
     <comment ref="I1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">cohort_year
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">Tahun angkatan masuk kuliah, empat digit. Kosongkan bila tidak diketahui.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">period_start
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">WAJIB DIISI. Tahun mulai kepengurusan, empat digit.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <family val="2"/>
+            <b val="1"/>
+            <color/>
+          </rPr>
+          <t xml:space="preserve">period_end
+</t>
+        </r>
+        <r>
+          <rPr>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <color indexed="81"/>
+            <sz val="9"/>
+          </rPr>
+          <t xml:space="preserve">WAJIB DIISI. Tahun akhir kepengurusan, empat digit.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -223,7 +289,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
   <si>
     <t>name</t>
   </si>
@@ -270,6 +336,33 @@
     <t>https://instagram.com/aulia</t>
   </si>
   <si>
+    <t>faculty</t>
+  </si>
+  <si>
+    <t>Fakultas Informatika</t>
+  </si>
+  <si>
+    <t>Fakultas Rekayasa Industri</t>
+  </si>
+  <si>
+    <t>study_program</t>
+  </si>
+  <si>
+    <t>S1 Informatika</t>
+  </si>
+  <si>
+    <t>S1 Sistem Informasi</t>
+  </si>
+  <si>
+    <t>cohort_year</t>
+  </si>
+  <si>
+    <t>2021</t>
+  </si>
+  <si>
+    <t>2022</t>
+  </si>
+  <si>
     <t>period_start</t>
   </si>
   <si>
@@ -363,7 +456,16 @@
     <t>Tautan lengkap profil Instagram, diawali https://.</t>
   </si>
   <si>
+    <t>Fakultas anggota.</t>
+  </si>
+  <si>
+    <t>Program studi anggota.</t>
+  </si>
+  <si>
     <t>angka</t>
+  </si>
+  <si>
+    <t>Tahun angkatan masuk kuliah, empat digit. Kosongkan bila tidak diketahui.</t>
   </si>
   <si>
     <t>Tahun mulai kepengurusan, empat digit.</t>
@@ -717,8 +819,11 @@
   <cols>
     <col customWidth="true" max="5" min="1" width="16"/>
     <col customWidth="true" max="6" min="6" width="19"/>
-    <col customWidth="true" max="7" min="7" width="18"/>
-    <col customWidth="true" max="9" min="8" width="16"/>
+    <col customWidth="true" max="7" min="7" width="16"/>
+    <col customWidth="true" max="8" min="8" width="19"/>
+    <col customWidth="true" max="9" min="9" width="17"/>
+    <col customWidth="true" max="10" min="10" width="18"/>
+    <col customWidth="true" max="12" min="11" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -740,14 +845,23 @@
       <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2">
@@ -773,10 +887,19 @@
         <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="I2" t="s">
-        <v>21</v>
+        <v>22</v>
+      </c>
+      <c r="J2" t="s">
+        <v>25</v>
+      </c>
+      <c r="K2" t="s">
+        <v>26</v>
+      </c>
+      <c r="L2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="3">
@@ -802,10 +925,19 @@
         <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" t="s">
-        <v>21</v>
+        <v>23</v>
+      </c>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" t="s">
+        <v>28</v>
+      </c>
+      <c r="L3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -825,71 +957,71 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
@@ -897,13 +1029,13 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C15" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16">
@@ -911,13 +1043,13 @@
         <v>3</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17">
@@ -925,13 +1057,13 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C17" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18">
@@ -939,13 +1071,13 @@
         <v>9</v>
       </c>
       <c r="B18" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19">
@@ -953,13 +1085,13 @@
         <v>11</v>
       </c>
       <c r="B19" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20">
@@ -967,13 +1099,13 @@
         <v>13</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21">
@@ -981,13 +1113,13 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22">
@@ -995,27 +1127,69 @@
         <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D23" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
         <v>50</v>
+      </c>
+      <c r="C26" t="s">
+        <v>61</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>